<commit_message>
feat(F-NAR-009): 126 atomiques EMO/FAM/JEU et ramifiées AUT-017–032
Ouvertures monde d’abord, chacune différente. Deux fichiers encore
incomplets (LEX.006-05, LEX.007-04) reportés. Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-03.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-03.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chloé est triste, deux fois</t>
+          <t>Sarah et le dessin mouillé</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Au jardin, une goutte mouille le soleil de Sarah. Elle dit qu'elle est triste. Elle demande un câlin. Plus tard, Nina part plus tôt. Sarah nomme encore la tristesse.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Chloé est dans le jardin avec maman. Son dessin a une tache d'eau. Chloé sent sa gorge serrée. Ses yeux sont mouillés. Je suis triste. Pleurer est permis. Pleurer permis. Chloé pleure un peu. Elle demande un câlin. Maman la serre. Le câlin est chaud. Chloé respire. Plus tard, à l'école, Lila part plus tôt. Chloé sent son ventre lourd. Elle se souvient. Elle dit à la maîtresse : je suis triste. Pleurer est permis. Chloé a les joues humides. Elle va vers maman, à la porte. Elle demande un câlin. Maman est là. Même leçon, autre lieu. Triste, on peut pleurer. On peut demander un câlin.</t>
+          <t>Une goutte pend au bec de l'arrosoir. La table du jardin est encore humide. Un galet tient une feuille de papier. Ça sent la menthe, tout près. Une abeille passe, puis plus. Les crayons jaunes attendent dans une boîte. Sarah, tu dessines le soleil ? Oui. Un grand soleil. Le papier est bien tenu. J'apporte le petit seau. En ce moment, Sarah dessine. Le crayon jaune frotte le papier. Un rond, puis des rayons. Il brille, maman. Il brille, oui. Maman arrose la menthe. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil... Parce que le dessin a une tache. Sarah sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Sarah pleure un peu. Les larmes sont chaudes sur ses joues. Je t'écoute, Sarah. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Sarah se blottit. Le câlin est chaud. Ça sent le savon de maman. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Sarah. Le câlin aide. Oui. Le câlin aide. Plus tard, près de l'école. Le gravier craque sous les chaussures. Un manteau sent encore la cour. Le portail est froid sous la main. Nina boutonne son manteau rouge. Je rentre plus tôt. Nina part, tout doucement. Sarah sent son ventre lourd. Elle se souvient du jardin. Je suis triste. Maman arrive à la porte. Tu es triste. C'est permis. Pleurer est permis. Sarah a les joues humides. Je veux un câlin. Viens. Un câlin. Maman la serre. Le câlin est chaud, encore. Bravo, Sarah. Tu as dit tes larmes. On peut demander un câlin. Au jardin, puis ici. Au jardin, c'était pareil. Sarah respire. Maman tient sa main.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,15 +1324,77 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Chloé est dans le jardin avec maman. Son dessin a une tache d'eau. Chloé sent sa gorge serrée. Ses yeux sont mouillés.
-narrateur|Je suis triste.
-maman|Pleurer est permis. Pleurer permis.
-narrateur|Chloé pleure un peu. Elle demande un câlin. Maman la serre. Le câlin est chaud. Chloé respire. Plus tard, à l'école, Lila part plus tôt. Chloé sent son ventre lourd. Elle se souvient. Elle dit à la maîtresse : je suis triste.
-maitresse|Pleurer est permis.
-narrateur|Chloé a les joues humides. Elle va vers maman, à la porte. Elle demande un câlin. Maman est là. Même leçon, autre lieu. Triste, on peut pleurer. On peut demander un câlin.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|Une goutte pend au bec de l'arrosoir.
+narrateur|La table du jardin est encore humide.
+narrateur|Un galet tient une feuille de papier.
+narrateur|Ça sent la menthe, tout près.
+narrateur|Une abeille passe, puis plus.
+narrateur|Les crayons jaunes attendent dans une boîte.
+maman|Sarah, tu dessines le soleil ?
+enfant-f|Oui. Un grand soleil.
+maman|Le papier est bien tenu.
+papa|J'apporte le petit seau.
+narrateur|En ce moment, Sarah dessine.
+narrateur|Le crayon jaune frotte le papier.
+narrateur|Un rond, puis des rayons.
+enfant-f|Il brille, maman.
+maman|Il brille, oui.
+narrateur|Maman arrose la menthe.
+narrateur|Une goutte tombe sur le dessin.
+narrateur|Le jaune coule un peu.
+enfant-f|Mon soleil...
+narrateur|Parce que le dessin a une tache.
+narrateur|Sarah sent sa gorge serrée.
+narrateur|Ses yeux deviennent chauds.
+narrateur|Une larme tombe.
+enfant-f|Je suis triste.
+maman|Tu es triste. C'est permis.
+maman|Pleurer est permis.
+narrateur|Sarah pleure un peu.
+narrateur|Les larmes sont chaudes sur ses joues.
+papa|Je t'écoute, Sarah.
+enfant-f|Je veux un câlin.
+maman|Viens. Un câlin.
+narrateur|Maman ouvre les bras.
+narrateur|Sarah se blottit.
+narrateur|Le câlin est chaud.
+narrateur|Ça sent le savon de maman.
+maman|Tu as dit : je suis triste.
+maman|Bravo. Tu as demandé un câlin.
+papa|Pleurer est permis, Sarah.
+enfant-f|Le câlin aide.
+maman|Oui. Le câlin aide.
+narrateur|Plus tard, près de l'école.
+narrateur|Le gravier craque sous les chaussures.
+narrateur|Un manteau sent encore la cour.
+narrateur|Le portail est froid sous la main.
+narrateur|Nina boutonne son manteau rouge.
+enfant-f|Je rentre plus tôt.
+narrateur|Nina part, tout doucement.
+narrateur|Sarah sent son ventre lourd.
+narrateur|Elle se souvient du jardin.
+enfant-f|Je suis triste.
+narrateur|Maman arrive à la porte.
+maman|Tu es triste. C'est permis.
+maman|Pleurer est permis.
+narrateur|Sarah a les joues humides.
+enfant-f|Je veux un câlin.
+maman|Viens. Un câlin.
+narrateur|Maman la serre.
+narrateur|Le câlin est chaud, encore.
+papa|Bravo, Sarah. Tu as dit tes larmes.
+papa|On peut demander un câlin.
+enfant-f|Au jardin, puis ici.
+maman|Au jardin, c'était pareil.
+narrateur|Sarah respire.
+narrateur|Maman tient sa main.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>jardin</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1345,7 +1419,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chloé est triste. Que peut-elle faire ?</t>
+          <t>Sarah est triste. Que peut-elle faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1505,7 +1579,7 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chloé est triste. Que peut-elle faire ?</t>
+          <t>narrateur|Sarah est triste. Que peut-elle faire ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1533,7 +1607,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chloé Je suis triste. Au jardin, puis à l'école. Un câlin a aidé.</t>
+          <t>Sarah essuie une joue avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin aide. Bravo. Tu as dit tes larmes. Tu veux encore un câlin ? Oui. Au jardin, puis ici. Maman la serre, sans se presser. Le portail reste froid, tout près.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1677,9 +1751,15 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chloé
-enfant-f|Je suis triste. Au jardin, puis à l'école.
-narrateur|Un câlin a aidé.</t>
+          <t>narrateur|Sarah essuie une joue avec sa manche.
+enfant-f|Je suis triste.
+maman|Oui. Et pleurer est permis.
+maman|Un câlin aide.
+papa|Bravo. Tu as dit tes larmes.
+papa|Tu veux encore un câlin ?
+enfant-f|Oui. Au jardin, puis ici.
+narrateur|Maman la serre, sans se presser.
+narrateur|Le portail reste froid, tout près.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1707,7 +1787,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chloé respire. Maman tient sa main.</t>
+          <t>Sarah respire, plus doucement. Le dessin reste dans le sac. On rentre quand tu es prête ? Encore ta main. On reste. Tu as bien demandé le câlin. C'est du bon travail. Je suis moins triste. Le câlin est encore là. Ils restent près du portail, tout calmes. Maman tient sa main.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1847,7 +1927,16 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Chloé respire. Maman tient sa main.</t>
+          <t>narrateur|Sarah respire, plus doucement.
+narrateur|Le dessin reste dans le sac.
+maman|On rentre quand tu es prête ?
+enfant-f|Encore ta main.
+papa|On reste. Tu as bien demandé le câlin.
+papa|C'est du bon travail.
+enfant-f|Je suis moins triste.
+maman|Le câlin est encore là.
+narrateur|Ils restent près du portail, tout calmes.
+narrateur|Maman tient sa main.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1875,7 +1964,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Sarah. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2015,7 +2104,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-f|J'ai dit : je suis triste.
+enfant-f|J'ai eu un câlin.
+maman|Pleurer est permis.
+papa|Bravo, Sarah.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2037,7 +2130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2075,6 +2168,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.002-03 Sarah et le dessin mouillé
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-03.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, puis porte de l'école</t>
+          <t>jardin, puis porte de l'école, table, arrosoir, galet, dessin, goutte, paillasson, menthe, manteau</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Nina, maman, papa</t>
+          <t>Sarah, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au jardin, une goutte mouille le soleil de Sarah. Elle dit qu'elle est triste. Elle demande un câlin. Plus tard, Nina part plus tôt. Sarah nomme encore la tristesse.</t>
+          <t>Sarah connaît la table du jardin. Sur le paillasson, un éclat de paillasson luit. Elle veut finir le soleil pour Nina, maintenant. Une goutte tombe. Sourire parti. Poitrine serrée. Papa s'accroupit. Elle dit je suis triste. Elle demande un câlin. Merci vécu. Deuxième ruse : Nina part plus tôt, le dessin est mouillé. Elle refuse de foncer. Un éclat de paillasson tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte pend au bec de l'arrosoir. La table du jardin est encore humide. Un galet tient une feuille de papier. Ça sent la menthe, tout près. Une abeille passe, puis plus. Les crayons jaunes attendent dans une boîte. Sarah, tu dessines le soleil ? Oui. Un grand soleil. Le papier est bien tenu. J'apporte le petit seau. En ce moment, Sarah dessine. Le crayon jaune frotte le papier. Un rond, puis des rayons. Il brille, maman. Il brille, oui. Maman arrose la menthe. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil... Parce que le dessin a une tache. Sarah sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Sarah pleure un peu. Les larmes sont chaudes sur ses joues. Je t'écoute, Sarah. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Sarah se blottit. Le câlin est chaud. Ça sent le savon de maman. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Sarah. Le câlin aide. Oui. Le câlin aide. Plus tard, près de l'école. Le gravier craque sous les chaussures. Un manteau sent encore la cour. Le portail est froid sous la main. Nina boutonne son manteau rouge. Je rentre plus tôt. Nina part, tout doucement. Sarah sent son ventre lourd. Elle se souvient du jardin. Je suis triste. Maman arrive à la porte. Tu es triste. C'est permis. Pleurer est permis. Sarah a les joues humides. Je veux un câlin. Viens. Un câlin. Maman la serre. Le câlin est chaud, encore. Bravo, Sarah. Tu as dit tes larmes. On peut demander un câlin. Au jardin, puis ici. Au jardin, c'était pareil. Sarah respire. Maman tient sa main.</t>
+          <t>Sarah connaît la table du jardin. Elle est à nous, Nina. Oui, Sarah. Nina pose un galet sur le papier. Il tient, papa. Tu le vois, le galet gris ? Oui, papa. Une goutte pend au bec de l'arrosoir. Elle brille, maman. Tu la vois, la goutte ? Oui, maman. Ça sent la menthe, près des genoux. Ça sent la menthe, papa. Tu la sens, la menthe tiède ? Oui. Sarah connaît ce jardin, ses recoins. Là, un coin brille autrement. Le paillasson de la porte est un peu dur. Il gratte, maman. Tu le sens, sous le doigt ? Oui, maman. Sur le paillasson, un éclat de paillasson luit. Il brille, Nina. Un petit point. Le soleil le touche. Un rayon glisse sur le bord. La table chauffe le papier. Il est chaud. Tu dessines le soleil, Sarah ? Oui, un grand soleil. Pour moi aussi ? Pour toi, Nina. En ce moment, Sarah dessine le soleil pour Nina. Je finis, maintenant ! Tout de suite ? Oui, papa. Le jaune frotte le papier. Un rond, puis des rayons. Il brille, Nina. Il est rond. Maman arrose la menthe, trop près. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil ! On souffle dessus ? Sarah souffle trop vite, tout de suite. Le jaune s'étale, plus large. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le papier. Je suis triste. Sarah pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Sarah ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je veux un câlin. Viens. Maman ouvre les bras. Sarah se blottit contre maman. Le câlin est chaud, près du cou. Ça sent le savon de maman. L'éclat de paillasson tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte pend au bec de l'arrosoir. La table du jardin est encore humide. Un galet tient une feuille de papier. Ça sent la menthe, tout près. Une abeille passe, puis plus. Les crayons jaunes attendent dans une boîte. Sarah, tu dessines le soleil ? Oui. Un grand soleil. Le papier est bien tenu. J'apporte le petit seau. En ce moment, Sarah dessine. Le crayon jaune frotte le papier. Un rond, puis des rayons. Il brille, maman. Il brille, oui. Maman arrose la menthe. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil... Parce que le dessin a une tache. Sarah sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Sarah pleure un peu. Les larmes sont chaudes sur ses joues. Je t'écoute, Sarah. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Sarah se blottit. Le câlin est chaud. Ça sent le savon de maman. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Sarah. Le câlin aide. Oui. Le câlin aide. Plus tard, près de l'école. Le gravier craque sous les chaussures. Un manteau sent encore la cour. Le portail est froid sous la main. Nina boutonne son manteau rouge. Je rentre plus tôt. Nina part, tout doucement. Sarah sent son ventre lourd. Elle se souvient du jardin. Je suis triste. Maman arrive à la porte. Tu es triste. C'est permis. Pleurer est permis. Sarah a les joues humides. Je veux un câlin. Viens. Un câlin. Maman la serre. Le câlin est chaud, encore. Bravo, Sarah. Tu as dit tes larmes. On peut demander un câlin. Au jardin, puis ici. Au jardin, c'était pareil. Sarah respire. Maman tient sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah connaît la table du jardin. Elle est à nous, Nina. Oui, Sarah. Nina pose un galet sur le papier. Il tient, papa. Tu le vois, le galet gris ? Oui, papa. Une goutte pend au bec de l'arrosoir. Elle brille, maman. Tu la vois, la goutte ? Oui, maman. Ça sent la menthe, près des genoux. Ça sent la menthe, papa. Tu la sens, la menthe tiède ? Oui. Sarah connaît ce jardin, ses recoins. Là, un coin brille autrement. Le paillasson de la porte est un peu dur. Il gratte, maman. Tu le sens, sous le doigt ? Oui, maman. Sur le paillasson, un &lt;emphasis level="moderate"&gt;éclat de paillasson&lt;/emphasis&gt; luit. Il brille, Nina. Un petit point. Le soleil le touche. Un rayon glisse sur le bord. La table chauffe le papier. Il est chaud. Tu dessines le soleil, Sarah ? Oui, un grand soleil. Pour moi aussi ? Pour toi, Nina. En ce moment, Sarah dessine le soleil pour Nina. Je finis, maintenant ! Tout de suite ? Oui, papa. Le jaune frotte le papier. Un rond, puis des rayons. Il brille, Nina. Il est rond. Maman arrose la menthe, trop près. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil ! On souffle dessus ? Sarah souffle trop vite, tout de suite. Le jaune s'étale, plus large. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le papier. Je suis triste. Sarah pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Sarah ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je veux un câlin. Viens. Maman ouvre les bras. Sarah se blottit contre maman. Le câlin est chaud, près du cou. Ça sent le savon de maman. L'éclat de paillasson tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Chloé est dans le jardin avec maman. Son dessin a une tache d'eau. Chloé sent sa gorge serrée. Ses yeux sont mouillés. Elle dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Maman dit : pleurer est permis. Pleurer permis. Chloé pleure un peu. Elle demande un câlin. Maman la serre. Le câlin est chaud. Chloé respire. Plus tard, à l'école, Lila part plus tôt. Chloé sent son ventre lourd. Elle se souvient. Elle dit à la maîtresse : je suis triste. La maîtresse dit : pleurer est permis. Chloé a les joues humides. Elle va vers maman, à la porte. Elle demande un câlin. Maman est là. Même leçon, autre lieu. Triste, on peut pleurer. On peut demander un câlin. [pause]</t>
+          <t>Sarah connaît la table du jardin. Elle est à nous, Nina. Oui, Sarah. Nina pose un galet sur le papier. Il tient, papa. Tu le vois, le galet gris ? Oui, papa. Une goutte pend au bec de l'arrosoir. Elle brille, maman. Tu la vois, la goutte ? Oui, maman. Ça sent la menthe, près des genoux. Ça sent la menthe, papa. Tu la sens, la menthe tiède ? Oui. Sarah connaît ce jardin, ses recoins. Là, un coin brille autrement. Le paillasson de la porte est un peu dur. Il gratte, maman. Tu le sens, sous le doigt ? Oui, maman. Sur le paillasson, un &lt;emphasis&gt;éclat de paillasson&lt;/emphasis&gt; luit. Il brille, Nina. Un petit point. Le soleil le touche. Un rayon glisse sur le bord. La table chauffe le papier. Il est chaud. Tu dessines le soleil, Sarah ? Oui, un grand soleil. Pour moi aussi ? Pour toi, Nina. En ce moment, Sarah dessine le soleil pour Nina. Je finis, maintenant ! Tout de suite ? Oui, papa. Le jaune frotte le papier. Un rond, puis des rayons. Il brille, Nina. Il est rond. Maman arrose la menthe, trop près. Une goutte tombe sur le dessin. Le jaune coule un peu. Mon soleil ! On souffle dessus ? Sarah souffle trop vite, tout de suite. Le jaune s'étale, plus large. Il part ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ses yeux deviennent chauds. Une larme tombe sur le papier. Je suis triste. Sarah pleure un peu, sans crier. Les larmes coulent sur ses joues. Tu as les yeux chauds, Sarah ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je veux un câlin. Viens. Maman ouvre les bras. Sarah se blottit contre maman. Le câlin est chaud, près du cou. Ça sent le savon de maman. L'éclat de paillasson tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>éclat de paillasson</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,73 +1321,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis tristesse; intensite=2; destinataire=enfant; sous_texte=elle_veut_finir_le_soleil_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte pend au bec de l'arrosoir.
-narrateur|La table du jardin est encore humide.
-narrateur|Un galet tient une feuille de papier.
-narrateur|Ça sent la menthe, tout près.
-narrateur|Une abeille passe, puis plus.
-narrateur|Les crayons jaunes attendent dans une boîte.
-maman|Sarah, tu dessines le soleil ?
-enfant-f|Oui. Un grand soleil.
-maman|Le papier est bien tenu.
-papa|J'apporte le petit seau.
-narrateur|En ce moment, Sarah dessine.
-narrateur|Le crayon jaune frotte le papier.
+          <t>narrateur|Sarah connaît la table du jardin.
+enfant-f|Elle est à nous, Nina.
+copine|Oui, Sarah.
+narrateur|Nina pose un galet sur le papier.
+enfant-f|Il tient, papa.
+papa|Tu le vois, le galet gris ?
+enfant-f|Oui, papa.
+narrateur|Une goutte pend au bec de l'arrosoir.
+copine|Elle brille, maman.
+maman|Tu la vois, la goutte ?
+copine|Oui, maman.
+narrateur|Ça sent la menthe, près des genoux.
+enfant-f|Ça sent la menthe, papa.
+papa|Tu la sens, la menthe tiède ?
+enfant-f|Oui.
+narrateur|Sarah connaît ce jardin, ses recoins.
+narrateur|Là, un coin brille autrement.
+narrateur|Le paillasson de la porte est un peu dur.
+enfant-f|Il gratte, maman.
+maman|Tu le sens, sous le doigt ?
+enfant-f|Oui, maman.
+narrateur|Sur le paillasson, un éclat de paillasson luit.
+enfant-f|Il brille, Nina.
+copine|Un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur le bord.
+narrateur|La table chauffe le papier.
+enfant-f|Il est chaud.
+maman|Tu dessines le soleil, Sarah ?
+enfant-f|Oui, un grand soleil.
+copine|Pour moi aussi ?
+enfant-f|Pour toi, Nina.
+narrateur|En ce moment, Sarah dessine le soleil pour Nina.
+enfant-f|Je finis, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Le jaune frotte le papier.
 narrateur|Un rond, puis des rayons.
-enfant-f|Il brille, maman.
-maman|Il brille, oui.
-narrateur|Maman arrose la menthe.
+enfant-f|Il brille, Nina.
+copine|Il est rond.
+narrateur|Maman arrose la menthe, trop près.
 narrateur|Une goutte tombe sur le dessin.
 narrateur|Le jaune coule un peu.
-enfant-f|Mon soleil...
-narrateur|Parce que le dessin a une tache.
-narrateur|Sarah sent sa gorge serrée.
+enfant-f|Mon soleil !
+copine|On souffle dessus ?
+narrateur|Sarah souffle trop vite, tout de suite.
+narrateur|Le jaune s'étale, plus large.
+enfant-f|Il part !
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+enfant-f|J'ai mal au ventre.
 narrateur|Ses yeux deviennent chauds.
-narrateur|Une larme tombe.
+narrateur|Une larme tombe sur le papier.
 enfant-f|Je suis triste.
-maman|Tu es triste. C'est permis.
-maman|Pleurer est permis.
-narrateur|Sarah pleure un peu.
-narrateur|Les larmes sont chaudes sur ses joues.
-papa|Je t'écoute, Sarah.
+narrateur|Sarah pleure un peu, sans crier.
+narrateur|Les larmes coulent sur ses joues.
+papa|Tu as les yeux chauds, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Sarah ?
+enfant-f|Un peu, maman.
 enfant-f|Je veux un câlin.
-maman|Viens. Un câlin.
+maman|Viens.
 narrateur|Maman ouvre les bras.
-narrateur|Sarah se blottit.
-narrateur|Le câlin est chaud.
+narrateur|Sarah se blottit contre maman.
+narrateur|Le câlin est chaud, près du cou.
 narrateur|Ça sent le savon de maman.
-maman|Tu as dit : je suis triste.
-maman|Bravo. Tu as demandé un câlin.
-papa|Pleurer est permis, Sarah.
-enfant-f|Le câlin aide.
-maman|Oui. Le câlin aide.
-narrateur|Plus tard, près de l'école.
-narrateur|Le gravier craque sous les chaussures.
-narrateur|Un manteau sent encore la cour.
-narrateur|Le portail est froid sous la main.
-narrateur|Nina boutonne son manteau rouge.
-enfant-f|Je rentre plus tôt.
-narrateur|Nina part, tout doucement.
-narrateur|Sarah sent son ventre lourd.
-narrateur|Elle se souvient du jardin.
-enfant-f|Je suis triste.
-narrateur|Maman arrive à la porte.
-maman|Tu es triste. C'est permis.
-maman|Pleurer est permis.
-narrateur|Sarah a les joues humides.
-enfant-f|Je veux un câlin.
-maman|Viens. Un câlin.
-narrateur|Maman la serre.
-narrateur|Le câlin est chaud, encore.
-papa|Bravo, Sarah. Tu as dit tes larmes.
-papa|On peut demander un câlin.
-enfant-f|Au jardin, puis ici.
-maman|Au jardin, c'était pareil.
-narrateur|Sarah respire.
-narrateur|Maman tient sa main.</t>
+narrateur|L'éclat de paillasson tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1424,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah est triste. Que peut-elle faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; est triste. Que peut-elle faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Chloé est &lt;emphasis&gt;triste&lt;/emphasis&gt;. Que peut-elle faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Sarah&lt;/emphasis&gt; est triste. Que peut-elle faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1454,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle peut dire je suis triste. Elle peut demander un câlin. Que fait Chloé ?</t>
+          <t>Elle peut dire je suis triste. Elle peut demander un câlin. Que fait Sarah ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1492,18 +1501,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1518,38 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>Sarah</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1558,28 +1567,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=sarah_est_triste_que_peut_elle_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Sarah est triste. Que peut-elle faire ?</t>
+          <t>narrateur|Sarah est triste.
+narrateur|Que peut-elle faire ?</t>
         </is>
       </c>
     </row>
@@ -1606,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah essuie une joue avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin aide. Bravo. Tu as dit tes larmes. Tu veux encore un câlin ? Oui. Au jardin, puis ici. Maman la serre, sans se presser. Le portail reste froid, tout près.</t>
+          <t>Sarah reste contre maman, un moment. Le soleil, maintenant. Les mots se bousculent dans sa bouche. Je le répare. Sarah avance la main, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le jardin, près de la table. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le câlin est tiède, sous les bras. Il est chaud. La poitrine de Sarah ralentit un peu. Les épaules se relèvent un peu. Tes joues sont mouillées, Sarah ? Un peu, maman. On laisse le jaune, sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le soleil est là, un peu mouillé. Il est à moi. Le galet tient le papier ? Oui, maman. Le ventre de Sarah se desserre. On va à l'école après ? Oui, papa. Sarah tient le tissu de maman. Je reste un peu. On le porte, le soleil ? Oui, Nina.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah essuie une joue avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin aide. Bravo. Tu as dit tes larmes. Tu veux encore un câlin ? Oui. Au jardin, puis ici. Maman la serre, sans se presser. Le portail reste froid, tout près.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah reste contre maman, un moment. Le soleil, maintenant. Les mots se bousculent dans sa bouche. Je le répare. Sarah avance la main, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le jardin, près de la table. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le &lt;emphasis level="moderate"&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. La poitrine de Sarah ralentit un peu. Les épaules se relèvent un peu. Tes joues sont mouillées, Sarah ? Un peu, maman. On laisse le jaune, sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le soleil est là, un peu mouillé. Il est à moi. Le galet tient le papier ? Oui, maman. Le ventre de Sarah se desserre. On va à l'école après ? Oui, papa. Sarah tient le tissu de maman. Je reste un peu. On le porte, le soleil ? Oui, Nina.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Chloé a dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Au jardin, puis à l'école. Un câlin a aidé. [pause]</t>
+          <t>Sarah reste contre maman, un moment. Le soleil, maintenant. Les mots se bousculent dans sa bouche. Je le répare. Sarah avance la main, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le dessin, un instant. Elle écoute le jardin, près de la table. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le &lt;emphasis&gt;câlin&lt;/emphasis&gt; est tiède, sous les bras. Il est chaud. La poitrine de Sarah ralentit un peu. Les épaules se relèvent un peu. Tes joues sont mouillées, Sarah ? Un peu, maman. On laisse le jaune, sans se presser ? Oui. Maman essuie une larme du pouce. Ça pique les yeux. Le soleil est là, un peu mouillé. Il est à moi. Le galet tient le papier ? Oui, maman. Le ventre de Sarah se desserre. On va à l'école après ? Oui, papa. Sarah tient le tissu de maman. Je reste un peu. On le porte, le soleil ? Oui, Nina. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1663,7 +1673,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1671,10 +1681,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1697,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>câlin</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1729,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1745,20 +1755,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_demande_un_calin_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah essuie une joue avec sa manche.
-enfant-f|Je suis triste.
-maman|Oui. Et pleurer est permis.
-maman|Un câlin aide.
-papa|Bravo. Tu as dit tes larmes.
-papa|Tu veux encore un câlin ?
-enfant-f|Oui. Au jardin, puis ici.
-narrateur|Maman la serre, sans se presser.
-narrateur|Le portail reste froid, tout près.</t>
+          <t>narrateur|Sarah reste contre maman, un moment.
+enfant-f|Le soleil, maintenant.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Je le répare.
+narrateur|Sarah avance la main, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le dessin, un instant.
+narrateur|Elle écoute le jardin, près de la table.
+papa|Tu restes un peu, Sarah ?
+enfant-f|Oui, papa.
+papa|Merci, Sarah.
+narrateur|Papa reste à la même hauteur.
+maman|Le câlin est tiède, sous les bras.
+enfant-f|Il est chaud.
+narrateur|La poitrine de Sarah ralentit un peu.
+narrateur|Les épaules se relèvent un peu.
+maman|Tes joues sont mouillées, Sarah ?
+enfant-f|Un peu, maman.
+papa|On laisse le jaune, sans se presser ?
+enfant-f|Oui.
+narrateur|Maman essuie une larme du pouce.
+enfant-f|Ça pique les yeux.
+copine|Le soleil est là, un peu mouillé.
+enfant-f|Il est à moi.
+maman|Le galet tient le papier ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Sarah se desserre.
+papa|On va à l'école après ?
+enfant-f|Oui, papa.
+narrateur|Sarah tient le tissu de maman.
+enfant-f|Je reste un peu.
+copine|On le porte, le soleil ?
+enfant-f|Oui, Nina.</t>
         </is>
       </c>
     </row>
@@ -1785,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah respire, plus doucement. Le dessin reste dans le sac. On rentre quand tu es prête ? Encore ta main. On reste. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près du portail, tout calmes. Maman tient sa main.</t>
+          <t>Près de la porte de l'école, le soir penche. Sarah tient le dessin, un peu mouillé. Pour Nina, papa. Tu le montres, Sarah ? Oui. Nina boutonne son manteau rouge. Je rentre plus tôt. Attends, Nina ! Sarah avance trop vite, tout de suite. Le dessin penche, trop humide. Il glisse ! Le jaune n'a pas séché. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute la porte, près du paillasson. Sur le paillasson, un éclat de paillasson luit. Là, sur le bord. On tient le papier ? Oui, papa. Nina s'éloigne d'un pas, puis deux. À demain, Sarah. À demain. Sarah veut courir, tout de suite. Puis elle lâche le pas. Je reste. Tu restes près de nous, Sarah ? Oui, maman. Je veux un câlin. Viens. Maman la serre, sans se presser. Le câlin est chaud, près du cou. Le dessin tient, Sarah ? Oui, un peu mouillé. Le manteau de Nina part au coin. Je l'ai vu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah respire, plus doucement. Le dessin reste dans le sac. On rentre quand tu es prête ? Encore ta main. On reste. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près du portail, tout calmes. Maman tient sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de la porte de l'école, le soir penche. Sarah tient le dessin, un peu mouillé. Pour Nina, papa. Tu le montres, Sarah ? Oui. Nina boutonne son manteau rouge. Je rentre plus tôt. Attends, Nina ! Sarah avance trop vite, tout de suite. Le dessin penche, trop humide. Il glisse ! Le jaune n'a pas séché. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute la porte, près du paillasson. Sur le paillasson, un &lt;emphasis level="moderate"&gt;éclat de paillasson&lt;/emphasis&gt; luit. Là, sur le bord. On tient le papier ? Oui, papa. Nina s'éloigne d'un pas, puis deux. À demain, Sarah. À demain. Sarah veut courir, tout de suite. Puis elle lâche le pas. Je reste. Tu restes près de nous, Sarah ? Oui, maman. Je veux un câlin. Viens. Maman la serre, sans se presser. Le câlin est chaud, près du cou. Le dessin tient, Sarah ? Oui, un peu mouillé. Le manteau de Nina part au coin. Je l'ai vu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Chloé respire. Maman tient sa &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Près de la porte de l'école, le soir penche. Sarah tient le dessin, un peu mouillé. Pour Nina, papa. Tu le montres, Sarah ? Oui. Nina boutonne son manteau rouge. Je rentre plus tôt. Attends, Nina ! Sarah avance trop vite, tout de suite. Le dessin penche, trop humide. Il glisse ! Le jaune n'a pas séché. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le dessin, un instant. Elle écoute la porte, près du paillasson. Sur le paillasson, un &lt;emphasis&gt;éclat de paillasson&lt;/emphasis&gt; luit. Là, sur le bord. On tient le papier ? Oui, papa. Nina s'éloigne d'un pas, puis deux. À demain, Sarah. À demain. Sarah veut courir, tout de suite. Puis elle lâche le pas. Je reste. Tu restes près de nous, Sarah ? Oui, maman. Je veux un câlin. Viens. Maman la serre, sans se presser. Le câlin est chaud, près du cou. Le dessin tient, Sarah ? Oui, un peu mouillé. Le manteau de Nina part au coin. Je l'ai vu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1842,7 +1879,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1850,10 +1887,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1876,30 +1913,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de paillasson</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1908,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1922,18 +1959,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=nina_part_plus_tot_le_dessin_est_mouille; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah respire, plus doucement.
-narrateur|Le dessin reste dans le sac.
-maman|On rentre quand tu es prête ?
-enfant-f|Encore ta main.
-papa|On reste. Tu as bien demandé le câlin.
-enfant-f|Je suis moins triste.
-maman|Le câlin est encore là.
-narrateur|Ils restent près du portail, tout calmes.
-narrateur|Maman tient sa main.</t>
+          <t>narrateur|Près de la porte de l'école, le soir penche.
+narrateur|Sarah tient le dessin, un peu mouillé.
+enfant-f|Pour Nina, papa.
+papa|Tu le montres, Sarah ?
+enfant-f|Oui.
+narrateur|Nina boutonne son manteau rouge.
+copine|Je rentre plus tôt.
+enfant-f|Attends, Nina !
+narrateur|Sarah avance trop vite, tout de suite.
+narrateur|Le dessin penche, trop humide.
+enfant-f|Il glisse !
+narrateur|Le jaune n'a pas séché.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le dessin, un instant.
+narrateur|Elle écoute la porte, près du paillasson.
+narrateur|Sur le paillasson, un éclat de paillasson luit.
+enfant-f|Là, sur le bord.
+papa|On tient le papier ?
+enfant-f|Oui, papa.
+narrateur|Nina s'éloigne d'un pas, puis deux.
+copine|À demain, Sarah.
+enfant-f|À demain.
+narrateur|Sarah veut courir, tout de suite.
+narrateur|Puis elle lâche le pas.
+enfant-f|Je reste.
+maman|Tu restes près de nous, Sarah ?
+enfant-f|Oui, maman.
+enfant-f|Je veux un câlin.
+maman|Viens.
+narrateur|Maman la serre, sans se presser.
+narrateur|Le câlin est chaud, près du cou.
+papa|Le dessin tient, Sarah ?
+enfant-f|Oui, un peu mouillé.
+maman|Le manteau de Nina part au coin.
+enfant-f|Je l'ai vu.</t>
         </is>
       </c>
     </row>
@@ -1960,17 +2031,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Sarah.</t>
+          <t>Ils restent près de la porte. Maman essuie un peu de jaune. Nina est partie, papa. Tu l'as vue, toi ? Oui, avec son manteau. On est bien, ici. Sarah tapote le papier du doigt. Il a une tache d'eau. Tu la vois, la tache ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent la menthe, un peu tiède. Et le savon, maman. Oui, dans l'air. On reste ici, Sarah ? Oui, papa. Le dessin reste contre Sarah. Un éclat de paillasson tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Sarah.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la porte. Maman essuie un peu de jaune. Nina est partie, papa. Tu l'as vue, toi ? Oui, avec son manteau. On est bien, ici. Sarah tapote le papier du doigt. Il a une tache d'eau. Tu la vois, la tache ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent la menthe, un peu tiède. Et le savon, maman. Oui, dans l'air. On reste ici, Sarah ? Oui, papa. Le dessin reste contre Sarah. Un &lt;emphasis level="moderate"&gt;éclat de paillasson&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la porte. Maman essuie un peu de jaune. Nina est partie, papa. Tu l'as vue, toi ? Oui, avec son manteau. On est bien, ici. Sarah tapote le papier du doigt. Il a une tache d'eau. Tu la vois, la tache ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent la menthe, un peu tiède. Et le savon, maman. Oui, dans l'air. On reste ici, Sarah ? Oui, papa. Le dessin reste contre Sarah. Un &lt;emphasis&gt;éclat de paillasson&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,18 +2088,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2037,12 +2108,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2122,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de paillasson</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2145,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,27 +2158,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis triste.
-enfant-f|J'ai eu un câlin.
-maman|Pleurer est permis.
-papa|Bravo, Sarah.</t>
+          <t>narrateur|Ils restent près de la porte.
+narrateur|Maman essuie un peu de jaune.
+enfant-f|Nina est partie, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, avec son manteau.
+maman|On est bien, ici.
+narrateur|Sarah tapote le papier du doigt.
+enfant-f|Il a une tache d'eau.
+maman|Tu la vois, la tache ?
+enfant-f|Oui, maman.
+papa|Le dessin est resté, Sarah.
+enfant-f|Oui, avec le soleil.
+narrateur|Ça sent la menthe, un peu tiède.
+enfant-f|Et le savon, maman.
+maman|Oui, dans l'air.
+papa|On reste ici, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le dessin reste contre Sarah.
+narrateur|Un éclat de paillasson tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2174,6 +2268,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>